<commit_message>
fix: 収束グラフを ScatterChart → LineChart に変更
ScatterChart は系列ごとに X-Y を独立ペアで扱うため、カテゴリ（日付）と
値の対応がずれて累計が増えていないのにグラフが下降する問題があった。
LineChart（折れ線グラフ）に変更し、X 軸をカテゴリ軸（日付文字列）として
正しく累積推移が描画されるよう修正。to_serial によるシリアル値変換も不要になった。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/bugs_export.xlsx
+++ b/mgmt/tracker/reports/bugs_export.xlsx
@@ -18,9 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -124,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -157,7 +155,6 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -254,12 +251,15 @@
       </tx>
     </title>
     <plotArea>
-      <scatterChart>
+      <lineChart>
+        <grouping val="standard"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>累計登録</v>
+            <strRef>
+              <f>'欠陥収束'!B1</f>
+            </strRef>
           </tx>
           <spPr>
             <a:ln w="20000">
@@ -270,30 +270,31 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
-            <size val="5"/>
+            <symbol val="none"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
-          <xVal>
+          <cat>
             <numRef>
               <f>'欠陥収束'!$A$2:$A$33</f>
             </numRef>
-          </xVal>
-          <yVal>
+          </cat>
+          <val>
             <numRef>
               <f>'欠陥収束'!$B$2:$B$33</f>
             </numRef>
-          </yVal>
+          </val>
         </ser>
         <ser>
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>対応累計</v>
+            <strRef>
+              <f>'欠陥収束'!C1</f>
+            </strRef>
           </tx>
           <spPr>
             <a:ln w="20000">
@@ -304,30 +305,31 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
-            <size val="5"/>
+            <symbol val="none"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
-          <xVal>
+          <cat>
             <numRef>
               <f>'欠陥収束'!$A$2:$A$33</f>
             </numRef>
-          </xVal>
-          <yVal>
+          </cat>
+          <val>
             <numRef>
               <f>'欠陥収束'!$C$2:$C$33</f>
             </numRef>
-          </yVal>
+          </val>
         </ser>
         <ser>
           <idx val="2"/>
           <order val="2"/>
           <tx>
-            <v>確認累計</v>
+            <strRef>
+              <f>'欠陥収束'!D1</f>
+            </strRef>
           </tx>
           <spPr>
             <a:ln w="20000">
@@ -338,37 +340,33 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
-            <size val="5"/>
+            <symbol val="none"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
-          <xVal>
+          <cat>
             <numRef>
               <f>'欠陥収束'!$A$2:$A$33</f>
             </numRef>
-          </xVal>
-          <yVal>
+          </cat>
+          <val>
             <numRef>
               <f>'欠陥収束'!$D$2:$D$33</f>
             </numRef>
-          </yVal>
+          </val>
         </ser>
         <axId val="10"/>
-        <axId val="20"/>
-      </scatterChart>
-      <valAx>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="46161"/>
-          <min val="46130"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -384,13 +382,13 @@
             </rich>
           </tx>
         </title>
-        <numFmt formatCode="YYYY-MM-DD" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="20"/>
-      </valAx>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
       <valAx>
-        <axId val="20"/>
+        <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
           <min val="0"/>
@@ -2325,8 +2323,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="n">
-        <v>46130</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
@@ -2339,8 +2339,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n">
-        <v>46131</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
@@ -2353,8 +2355,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
-        <v>46132</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
       </c>
       <c r="B4" t="n">
         <v>2</v>
@@ -2367,8 +2371,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
-        <v>46133</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
       </c>
       <c r="B5" t="n">
         <v>2</v>
@@ -2381,8 +2387,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
-        <v>46134</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
       </c>
       <c r="B6" t="n">
         <v>2</v>
@@ -2395,8 +2403,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
-        <v>46135</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
@@ -2409,8 +2419,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
-        <v>46136</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
       </c>
       <c r="B8" t="n">
         <v>4</v>
@@ -2423,8 +2435,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
-        <v>46137</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
       </c>
       <c r="B9" t="n">
         <v>6</v>
@@ -2437,8 +2451,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
-        <v>46138</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
       </c>
       <c r="B10" t="n">
         <v>12</v>
@@ -2451,8 +2467,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n">
-        <v>46139</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
       </c>
       <c r="B11" t="n">
         <v>13</v>
@@ -2465,8 +2483,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
-        <v>46140</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
       </c>
       <c r="B12" t="n">
         <v>13</v>
@@ -2479,8 +2499,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n">
-        <v>46141</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
       </c>
       <c r="B13" t="n">
         <v>13</v>
@@ -2493,8 +2515,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
-        <v>46142</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
@@ -2507,8 +2531,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n">
-        <v>46143</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
       </c>
       <c r="B15" t="n">
         <v>13</v>
@@ -2521,8 +2547,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
-        <v>46144</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
       </c>
       <c r="B16" t="n">
         <v>14</v>
@@ -2535,8 +2563,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n">
-        <v>46145</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
       </c>
       <c r="B17" t="n">
         <v>14</v>
@@ -2549,8 +2579,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
-        <v>46146</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
       </c>
       <c r="B18" t="n">
         <v>14</v>
@@ -2563,8 +2595,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n">
-        <v>46147</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
       </c>
       <c r="B19" t="n">
         <v>14</v>
@@ -2577,8 +2611,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n">
-        <v>46148</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
       </c>
       <c r="B20" t="n">
         <v>14</v>
@@ -2591,8 +2627,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n">
-        <v>46149</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
       </c>
       <c r="B21" t="n">
         <v>14</v>
@@ -2605,8 +2643,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n">
-        <v>46150</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
       </c>
       <c r="B22" t="n">
         <v>14</v>
@@ -2619,8 +2659,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n">
-        <v>46151</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
       </c>
       <c r="B23" t="n">
         <v>14</v>
@@ -2633,8 +2675,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
-        <v>46152</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
       </c>
       <c r="B24" t="n">
         <v>14</v>
@@ -2647,8 +2691,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
-        <v>46153</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
       </c>
       <c r="B25" t="n">
         <v>14</v>
@@ -2661,8 +2707,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
-        <v>46154</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
       </c>
       <c r="B26" t="n">
         <v>14</v>
@@ -2675,8 +2723,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n">
-        <v>46155</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
       </c>
       <c r="B27" t="n">
         <v>14</v>
@@ -2689,8 +2739,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
-        <v>46156</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
       </c>
       <c r="B28" t="n">
         <v>14</v>
@@ -2703,8 +2755,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n">
-        <v>46157</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="B29" t="n">
         <v>14</v>
@@ -2717,8 +2771,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n">
-        <v>46158</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
       </c>
       <c r="B30" t="n">
         <v>14</v>
@@ -2731,8 +2787,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n">
-        <v>46159</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
       </c>
       <c r="B31" t="n">
         <v>14</v>
@@ -2745,8 +2803,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n">
-        <v>46160</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
       </c>
       <c r="B32" t="n">
         <v>14</v>
@@ -2759,8 +2819,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n">
-        <v>46161</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
       </c>
       <c r="B33" t="n">
         <v>14</v>

</xml_diff>